<commit_message>
Fase 6 (v2): columnas Log_, atípicos identificados por país y columna atipico
</commit_message>
<xml_diff>
--- a/diccionario_variables.xlsx
+++ b/diccionario_variables.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -764,35 +764,109 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Log_MOR / Log_CAPR / Log_ROA / Log_CRED</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Logaritmo en base 10 de cada variable; en el modelo log-log los coeficientes son elasticidades</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>log10(%)</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>mensual</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>03_limpieza_datos.py</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>origen_MOR / origen_CAPR / origen_ROA / origen_CRED</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Cómo se obtuvo cada dato: FMI_mensual_observado, FMI_trimestral_observado, BM_GFDD_anual_empalmado, BM_WDI_anual_observado, interpolado_lineal o imputado_media</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>texto</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D11" t="inlineStr">
         <is>
           <t>mensual</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>03_limpieza_datos.py</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>atipico</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1 si alguna variable de la fila es atípica dentro de su país (regla de Tukey); 0 si no</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>0/1</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>mensual</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>03_limpieza_datos.py</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
         <is>
           <t>2025-12</t>
         </is>

</xml_diff>